<commit_message>
fix: sanitize worksheet names to remove invalid Excel characters
Co-authored-by: lirantal <316371+lirantal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/__tests__/Fixtures/sample.xlsx
+++ b/__tests__/Fixtures/sample.xlsx
@@ -4,8 +4,8 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Question 1?" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Question 2?" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="Question 1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Question 2" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>

</xml_diff>

<commit_message>
chore: modernize CI workflows (#48)
* chore: modernize CI workflows

* fix: sanitize worksheet names to remove invalid Excel characters

Co-authored-by: lirantal <316371+lirantal@users.noreply.github.com>

* fix: revert package-lock.json to working v1 format compatible with npm ci

Co-authored-by: lirantal <316371+lirantal@users.noreply.github.com>

---------

Co-authored-by: copilot-swe-agent[bot] <198982749+Copilot@users.noreply.github.com>
Co-authored-by: lirantal <316371+lirantal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/__tests__/Fixtures/sample.xlsx
+++ b/__tests__/Fixtures/sample.xlsx
@@ -4,8 +4,8 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Question 1?" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Question 2?" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="Question 1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Question 2" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>

</xml_diff>